<commit_message>
chore: se actualiza la normalizacion
</commit_message>
<xml_diff>
--- a/02-Diseño/06-Normalizacion de datos/Normalizacion de datos.xlsx
+++ b/02-Diseño/06-Normalizacion de datos/Normalizacion de datos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/65771bf9c1e7ace5/Documents/Proyecto.GAE/Normalizacion de datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{9158158B-4532-4637-840F-AEDD12EE10E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C191E042-CC6C-4DB5-8DC7-7744C1853EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{4E6CDCF0-C4CD-4E29-915A-96AFCE44D247}"/>
   </bookViews>
@@ -450,12 +450,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -522,7 +534,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -538,13 +550,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -881,82 +900,82 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="G2" s="6" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="G2" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="J2" s="6" t="s">
+      <c r="H2" s="7"/>
+      <c r="J2" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="K2" s="6"/>
-      <c r="M2" s="6" t="s">
+      <c r="K2" s="7"/>
+      <c r="M2" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="A3" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="C3" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="M3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="N3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="O3" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="P3" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="Q3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="R3" s="1" t="s">
+      <c r="R3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="S3" s="1" t="s">
+      <c r="S3" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="T3" s="1" t="s">
+      <c r="T3" s="8" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1122,68 +1141,68 @@
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="F9" s="6" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="F9" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="G9" s="6"/>
-      <c r="I9" s="6" t="s">
+      <c r="G9" s="7"/>
+      <c r="I9" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="B10" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F10" s="2" t="s">
+      <c r="D10" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="K10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="M10" s="2" t="s">
+      <c r="K10" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="M10" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="N10" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O10" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="P10" s="2" t="s">
+      <c r="P10" s="9" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1272,78 +1291,78 @@
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="E16" s="6" t="s">
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="E16" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="I16" s="6" t="s">
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="I16" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="J16" s="6"/>
-      <c r="L16" s="6" t="s">
+      <c r="J16" s="7"/>
+      <c r="L16" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="M16" s="6"/>
-      <c r="N16" s="6"/>
-      <c r="O16" s="6"/>
-      <c r="P16" s="6"/>
-      <c r="Q16" s="6"/>
-      <c r="R16" s="6"/>
-      <c r="S16" s="6"/>
+      <c r="M16" s="7"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
+      <c r="Q16" s="7"/>
+      <c r="R16" s="7"/>
+      <c r="S16" s="7"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E17" s="2" t="s">
+      <c r="B17" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="G17" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="I17" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="J17" s="2" t="s">
+      <c r="J17" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="L17" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="M17" s="2" t="s">
+      <c r="M17" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="N17" s="2" t="s">
+      <c r="N17" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="O17" s="2" t="s">
+      <c r="O17" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="P17" s="2" t="s">
+      <c r="P17" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="Q17" s="2" t="s">
+      <c r="Q17" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="R17" s="2" t="s">
+      <c r="R17" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="S17" s="2" t="s">
+      <c r="S17" s="9" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1610,11 +1629,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A16:C16"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="I16:J16"/>
-    <mergeCell ref="L16:S16"/>
-    <mergeCell ref="L24:R24"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="J2:K2"/>
@@ -1622,6 +1636,11 @@
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="I9:P9"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="L16:S16"/>
+    <mergeCell ref="L24:R24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1635,57 +1654,58 @@
     <col min="1" max="1" width="13.26953125" customWidth="1"/>
     <col min="4" max="4" width="13.1796875" customWidth="1"/>
     <col min="6" max="6" width="13.453125" customWidth="1"/>
+    <col min="11" max="11" width="14.36328125" customWidth="1"/>
     <col min="14" max="14" width="13.453125" customWidth="1"/>
     <col min="15" max="15" width="15.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="F2" s="7" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="F2" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="G2" s="9"/>
-      <c r="H2" s="8"/>
-      <c r="J2" s="7" t="s">
+      <c r="G2" s="11"/>
+      <c r="H2" s="12"/>
+      <c r="J2" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="K2" s="9"/>
-      <c r="L2" s="8"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="12"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="9" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1809,82 +1829,82 @@
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="G10" s="6" t="s">
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="G10" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="H10" s="6"/>
-      <c r="J10" s="6" t="s">
+      <c r="H10" s="7"/>
+      <c r="J10" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="N10" s="6" t="s">
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="N10" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7"/>
+      <c r="R10" s="7"/>
+      <c r="S10" s="7"/>
+      <c r="T10" s="7"/>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J11" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="K11" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="L11" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="N11" s="2" t="s">
+      <c r="L11" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="N11" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="O11" s="2" t="s">
+      <c r="O11" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="P11" s="2" t="s">
+      <c r="P11" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="Q11" s="2" t="s">
+      <c r="Q11" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="R11" s="2" t="s">
+      <c r="R11" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="S11" s="2" t="s">
+      <c r="S11" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="T11" s="2" t="s">
+      <c r="T11" s="9" t="s">
         <v>47</v>
       </c>
     </row>
@@ -2180,16 +2200,16 @@
       <c r="H18" s="2">
         <v>3</v>
       </c>
-      <c r="N18" s="7" t="s">
+      <c r="N18" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="O18" s="8"/>
-      <c r="Q18" s="6" t="s">
+      <c r="O18" s="12"/>
+      <c r="Q18" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="R18" s="6"/>
-      <c r="S18" s="6"/>
-      <c r="T18" s="6"/>
+      <c r="R18" s="7"/>
+      <c r="S18" s="7"/>
+      <c r="T18" s="7"/>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
@@ -2213,22 +2233,22 @@
       <c r="H19" s="2">
         <v>3</v>
       </c>
-      <c r="N19" s="2" t="s">
+      <c r="N19" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="O19" s="2" t="s">
+      <c r="O19" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="Q19" s="2" t="s">
+      <c r="Q19" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="R19" s="2" t="s">
+      <c r="R19" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="S19" s="2" t="s">
+      <c r="S19" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="T19" s="2" t="s">
+      <c r="T19" s="9" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2432,46 +2452,46 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="G2" s="6" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="G2" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="E3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I3" s="2" t="s">
+      <c r="H3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="I3" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="9" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2568,32 +2588,32 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J11" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="K11" s="9" t="s">
         <v>100</v>
       </c>
     </row>

</xml_diff>